<commit_message>
Legend: document Milestones basis; README: gids are for the 8 data tabs
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/FundED-data-template.xlsx
+++ b/data/FundED-data-template.xlsx
@@ -2594,7 +2594,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D15"/>
+  <dimension ref="A1:D16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2801,96 +2801,100 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>date</t>
+          <t>basis</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>ISO date</t>
+          <t>What kind of claim the milestone is</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>YYYY-MM-DD</t>
+          <t>fact | requirement | estimate | interpretation</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Engage</t>
+          <t>Milestones</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>basis</t>
+          <t>date</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>What kind of claim the venue is</t>
+          <t>ISO date</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>fact | requirement | estimate | interpretation</t>
+          <t>YYYY-MM-DD</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Inquiries</t>
+          <t>Engage</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>status</t>
+          <t>basis</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Did the authority answer the question?</t>
+          <t>What kind of claim the venue is</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>answered | partial | unanswered</t>
+          <t>fact | requirement | estimate | interpretation</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Sources</t>
+          <t>Inquiries</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>source_id</t>
+          <t>status</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Referenced by every *_source_id column. Add the document here first.</t>
-        </is>
-      </c>
-      <c r="D13" s="2" t="inlineStr"/>
+          <t>Did the authority answer the question?</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>answered | partial | unanswered</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>(all)</t>
+          <t>Sources</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>*_id</t>
+          <t>source_id</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Lowercase letters and digits and dashes only. No spaces.</t>
+          <t>Referenced by every *_source_id column. Add the document here first.</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr"/>
@@ -2903,15 +2907,33 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
+          <t>*_id</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>Lowercase letters and digits and dashes only. No spaces.</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>(all)</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
           <t>blank cell</t>
         </is>
       </c>
-      <c r="C15" s="2" t="inlineStr">
+      <c r="C16" s="2" t="inlineStr">
         <is>
           <t>Leave blank when unknown. Never type TBD or ?.</t>
         </is>
       </c>
-      <c r="D15" s="2" t="inlineStr"/>
+      <c r="D16" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Oakridge depth: short answer, time scale, money picture, asks, open questions
Understand: a three-line short answer with one countdown; a proportional
axis from the April 2026 email to the planned 2029 finish; nested funding
bars ($80M bond, $31M Refresh, HVAC unpriced); a why-this-track line.
Act: engage venues sorted soonest-first with closing-date chips and a
ready-to-say ask with copy button; inquiries gain an "open" status for
questions nobody has asked yet.

Data model: Needs why_track fields; Engage date, deadline, ask; Inquiries
why and open status (date optional); new Funding tab (amount, parent_id).
Sheet, template builder, Legend, sync, tests, and Playwright spec updated.
Countdowns compute at build time; pin with FUNDED_AS_OF=YYYY-MM-DD.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/FundED-data-template.xlsx
+++ b/data/FundED-data-template.xlsx
@@ -14,8 +14,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Milestones" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Engage" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inquiries" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Legend" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Funding" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Legend" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -598,6 +599,496 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D23"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="41" customWidth="1" min="2" max="2"/>
+    <col width="60" customWidth="1" min="3" max="3"/>
+    <col width="48" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>tab</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>column</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>meaning</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>allowed_values</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Tracks</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>track_id</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Short id for the track (lowercase-dashes)</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Tracks</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>verification</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Has an APS contact confirmed this track's stages and deciders?</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>draft | documented | confirmed</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Stages</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>order</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Position of the stage within its track (1 = first)</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>whole number</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Stages</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>basis</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>What kind of claim the stage is</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>fact | requirement | estimate | interpretation</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Schools</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>live = every claim must have a source or the site will not build; draft = warnings only</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>live | draft</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Needs</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>current_stage_id</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Must be a stage_id that belongs to the need's track_id</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Needs</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>stage_basis / cost_basis / window_basis</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>What kind of claim each is</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>fact | requirement | estimate | interpretation</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Needs</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>why_track</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>One sentence on why the need sits on this track and not a faster one; shown under the pipeline</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Milestones</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Exactly one milestone per need must be next</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>done | next | later</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Milestones</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>basis</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>What kind of claim the milestone is</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>fact | requirement | estimate | interpretation</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Milestones</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>date</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>ISO date</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>YYYY-MM-DD</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Engage</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>basis</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>What kind of claim the venue is</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>fact | requirement | estimate | interpretation</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>Engage</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>date</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>ISO date the venue happens (a meeting, an election)</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>YYYY-MM-DD</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>Engage</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>deadline</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>ISO date the sign-up or application closes; venues sort by this when present</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>YYYY-MM-DD</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>Engage</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>ask</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>The specific question to put to this venue; shown with a copy button</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>Inquiries</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>open = a question no one has asked yet (leave date blank); the rest need a date</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>open | answered | partial | unanswered</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>Inquiries</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>why</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>Why the question matters or why it is still open</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>Funding</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>amount</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>Whole dollars, digits only (80000000). Leave blank when no source prices it separately.</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>number</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>Funding</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>parent_id</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>The funding_id this amount sits inside (same need). Blank for the top-level total.</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>Sources</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>source_id</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>Referenced by every *_source_id column. Add the document here first.</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>(all)</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>*_id</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>Lowercase letters and digits and dashes only. No spaces.</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>(all)</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>blank cell</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>Leave blank when unknown. Never type TBD or ?.</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -1314,7 +1805,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O2"/>
+  <dimension ref="A1:R2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -1332,6 +1823,9 @@
     <col width="21" customWidth="1" min="13" max="13"/>
     <col width="14" customWidth="1" min="14" max="14"/>
     <col width="18" customWidth="1" min="15" max="15"/>
+    <col width="60" customWidth="1" min="16" max="16"/>
+    <col width="17" customWidth="1" min="17" max="17"/>
+    <col width="21" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1410,6 +1904,21 @@
           <t>window_source_id</t>
         </is>
       </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>why_track</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>why_track_basis</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>why_track_source_id</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -1487,9 +1996,24 @@
           <t>cip-fy27-36</t>
         </is>
       </c>
+      <c r="P2" s="2" t="inlineStr">
+        <is>
+          <t>A whole-system HVAC replacement is a capital project: the School Board lists it in the 10-year CIP and funds it through County bonds, so it waits for the bond cycle. We found no dollar cutoff in any APS document that would move it to the faster maintenance (MC/MM) budget.</t>
+        </is>
+      </c>
+      <c r="Q2" s="2" t="inlineStr">
+        <is>
+          <t>interpretation</t>
+        </is>
+      </c>
+      <c r="R2" s="2" t="inlineStr">
+        <is>
+          <t>cip-fy27-36</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <dataValidations count="9">
+  <dataValidations count="11">
     <dataValidation sqref="B2:B500" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Unknown reference" error="Must match an id already listed on Schools" type="list">
       <formula1>=Schools!$A$2:$A$500</formula1>
     </dataValidation>
@@ -1515,6 +2039,12 @@
       <formula1>"fact,requirement,estimate,interpretation"</formula1>
     </dataValidation>
     <dataValidation sqref="O2:O500" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Unknown reference" error="Must match an id already listed on Sources" type="list">
+      <formula1>=Sources!$A$2:$A$500</formula1>
+    </dataValidation>
+    <dataValidation sqref="Q2:Q500" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Not an allowed value" error="Use one of: fact, requirement, estimate, interpretation" type="list">
+      <formula1>"fact,requirement,estimate,interpretation"</formula1>
+    </dataValidation>
+    <dataValidation sqref="R2:R500" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Unknown reference" error="Must match an id already listed on Sources" type="list">
       <formula1>=Sources!$A$2:$A$500</formula1>
     </dataValidation>
   </dataValidations>
@@ -1849,17 +2379,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H6"/>
+  <dimension ref="A1:K7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="21" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
-    <col width="60" customWidth="1" min="3" max="3"/>
+    <col width="51" customWidth="1" min="3" max="3"/>
     <col width="60" customWidth="1" min="4" max="4"/>
-    <col width="60" customWidth="1" min="5" max="5"/>
-    <col width="60" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="24" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="60" customWidth="1" min="7" max="7"/>
+    <col width="60" customWidth="1" min="8" max="8"/>
+    <col width="60" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="25" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1885,20 +2418,35 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
+          <t>date</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>deadline</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
           <t>how</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>ask</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>url</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>basis</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>source_id</t>
         </is>
@@ -1907,7 +2455,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>oakridge-sb-comment</t>
+          <t>oakridge-sb-oct8</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -1917,39 +2465,54 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>School Board meeting public comment</t>
+          <t>School Board meeting, Oct 8, 2026</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Regular meetings, generally 7 p.m. at the Syphax Education Center</t>
+          <t>Thursday, 7 p.m., Syphax Education Center, 2110 Washington Blvd</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Online speaker form opens four business days before and closes 4 p.m. the day before; max 30 speakers x 2 minutes</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>Sign up to speak: the online form opens Oct 2 (four business days before) and closes Oct 7 at 4 p.m. Two minutes per speaker, first 30 speakers.</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>If Question 4 passes on Nov 3, when does design for the Oakridge HVAC replacement start, and what is the plan for hot classrooms before construction begins in summer 2027?</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
           <t>https://www.apsva.us/arlington-school-board/school-board-meetings/sign-up-to-speak/</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
-        <is>
-          <t>requirement</t>
-        </is>
-      </c>
-      <c r="H2" s="2" t="inlineStr">
-        <is>
-          <t>aps-sign-up-to-speak</t>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>fact</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>aps-sb-meetings-2026-27</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>oakridge-ws-mcmm</t>
+          <t>oakridge-sb-oct22</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
@@ -1959,39 +2522,54 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>School Board work session on Facilities (Maintenance / Work Orders / MCMM)</t>
+          <t>School Board meeting, Oct 22, 2026</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 1:00-2:30 p.m.</t>
+          <t>Thursday, 7 p.m., Syphax Education Center, 2110 Washington Blvd</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Observe</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>https://www.apsva.us/post/september-schedule-of-board-meetings-work-sessions-and-advisory-council-and-committee-meetings-4/</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
+          <t>Sign up to speak: the online form opens Oct 16 and closes Oct 21 at 4 p.m. Two minutes per speaker, first 30 speakers.</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>If Question 4 fails, what happens to the Oakridge Refresh, and would the HVAC replacement move to the maintenance (MC/MM) budget or wait for the next bond?</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>https://www.apsva.us/arlington-school-board/school-board-meetings/sign-up-to-speak/</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
           <t>fact</t>
         </is>
       </c>
-      <c r="H3" s="2" t="inlineStr">
-        <is>
-          <t>aps-sept-2026-schedule</t>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>aps-sb-meetings-2026-27</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>oakridge-ws-fy28</t>
+          <t>oakridge-ccpta-oct21</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
@@ -2001,39 +2579,50 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>School Board work session on FY 2028 Budget Direction</t>
+          <t>County Council of PTAs (CCPTA) meeting</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29 10:45 a.m.-12:15 p.m.</t>
+          <t>Wednesday, Oct 21, 2026, 7 p.m., via Zoom</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Observe</t>
-        </is>
-      </c>
-      <c r="F4" s="2" t="inlineStr">
-        <is>
-          <t>https://www.apsva.us/post/september-schedule-of-board-meetings-work-sessions-and-advisory-council-and-committee-meetings-4/</t>
-        </is>
-      </c>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr"/>
       <c r="G4" s="2" t="inlineStr">
         <is>
+          <t>Open to PTA delegates only: ask your school PTA's CCPTA delegate to raise the need</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>Which other schools are waiting on the same Nov 3 bond, and can CCPTA ask APS for one written timeline per school?</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>https://www.arlingtonccpta.org/</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
           <t>fact</t>
         </is>
       </c>
-      <c r="H4" s="2" t="inlineStr">
-        <is>
-          <t>aps-sept-2026-schedule</t>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>ccpta-2026-27</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>oakridge-vote</t>
+          <t>oakridge-advisory</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
@@ -2043,39 +2632,46 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>General election Question 4</t>
+          <t>APS advisory councils (2026-27)</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>2026-11-03</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>Vote on the $80M school bond</t>
-        </is>
-      </c>
+          <t>Applications through Oct 31, 2026</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr"/>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>https://www.arlingtonva.us/Government/Programs/Budget-Finance/Bonds/2026-Bond-Referenda</t>
+          <t>2026-10-31</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
+          <t>Apply to a new advisory council</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr"/>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>https://www.apsva.us/post/september-schedule-of-board-meetings-work-sessions-and-advisory-council-and-committee-meetings-4/</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
           <t>fact</t>
         </is>
       </c>
-      <c r="H5" s="2" t="inlineStr">
-        <is>
-          <t>county-bond-2026</t>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
+          <t>aps-sept-2026-schedule</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>oakridge-advisory</t>
+          <t>oakridge-vote</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
@@ -2085,32 +2681,84 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>APS advisory councils (2026-27)</t>
+          <t>General election, Question 4</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Applications through 2026-10-31</t>
+          <t>Tuesday, Nov 3, 2026</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Apply to a new advisory council</t>
-        </is>
-      </c>
-      <c r="F6" s="2" t="inlineStr">
-        <is>
-          <t>https://www.apsva.us/post/september-schedule-of-board-meetings-work-sessions-and-advisory-council-and-committee-meetings-4/</t>
-        </is>
-      </c>
+          <t>2026-11-03</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr"/>
       <c r="G6" s="2" t="inlineStr">
         <is>
+          <t>Vote on the $80M school bond. Question 4 names the Oakridge Refresh.</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr"/>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>https://www.arlingtonva.us/Government/Programs/Budget-Finance/Bonds/2026-Bond-Referenda</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
           <t>fact</t>
         </is>
       </c>
-      <c r="H6" s="2" t="inlineStr">
-        <is>
-          <t>aps-sept-2026-schedule</t>
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t>county-bond-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>oakridge-sb-comment</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>oakridge-hvac</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>School Board meeting public comment (any meeting)</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>Regular meetings, generally 7 p.m. at the Syphax Education Center</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr"/>
+      <c r="F7" s="2" t="inlineStr"/>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>Online speaker form opens four business days before and closes 4 p.m. the day before; max 30 speakers x 2 minutes</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr"/>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>https://www.apsva.us/arlington-school-board/school-board-meetings/sign-up-to-speak/</t>
+        </is>
+      </c>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>requirement</t>
+        </is>
+      </c>
+      <c r="K7" s="2" t="inlineStr">
+        <is>
+          <t>aps-sign-up-to-speak</t>
         </is>
       </c>
     </row>
@@ -2119,10 +2767,10 @@
     <dataValidation sqref="B2:B500" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Unknown reference" error="Must match an id already listed on Needs" type="list">
       <formula1>=Needs!$A$2:$A$500</formula1>
     </dataValidation>
-    <dataValidation sqref="G2:G500" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Not an allowed value" error="Use one of: fact, requirement, estimate, interpretation" type="list">
+    <dataValidation sqref="J2:J500" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Not an allowed value" error="Use one of: fact, requirement, estimate, interpretation" type="list">
       <formula1>"fact,requirement,estimate,interpretation"</formula1>
     </dataValidation>
-    <dataValidation sqref="H2:H500" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Unknown reference" error="Must match an id already listed on Sources" type="list">
+    <dataValidation sqref="K2:K500" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Unknown reference" error="Must match an id already listed on Sources" type="list">
       <formula1>=Sources!$A$2:$A$500</formula1>
     </dataValidation>
   </dataValidations>
@@ -2136,18 +2784,19 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I2"/>
+  <dimension ref="A1:J4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="39" customWidth="1" min="4" max="4"/>
     <col width="60" customWidth="1" min="5" max="5"/>
-    <col width="15" customWidth="1" min="6" max="6"/>
-    <col width="60" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="15" customWidth="1" min="9" max="9"/>
+    <col width="60" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="60" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="18" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2178,20 +2827,25 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
+          <t>why</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
           <t>response_date</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>response_summary</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>status</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>source_id</t>
         </is>
@@ -2223,22 +2877,103 @@
           <t>What is the plan to make my children's school safe for learning over the next two months?</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="F2" s="2" t="inlineStr"/>
+      <c r="G2" s="2" t="inlineStr">
         <is>
           <t>2026-04-16</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="H2" s="2" t="inlineStr">
         <is>
           <t>Copied the school principal, who will work closely to monitor the situation.</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="I2" s="2" t="inlineStr">
         <is>
           <t>partial</t>
         </is>
       </c>
-      <c r="I2" s="2" t="inlineStr">
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>email-2026-04</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>q-if-bond-fails</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>oakridge-hvac</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr"/>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>APS Facilities and Operations</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>If Question 4 fails on Nov 3, what happens to the Oakridge Refresh, and does the HVAC replacement move to the maintenance budget?</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>No document says. The County notes the School Board may reallocate bond funds among CIP projects, and nothing names Oakridge either way.</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr"/>
+      <c r="H3" s="2" t="inlineStr"/>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>county-bond-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>q-interim-plan</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>oakridge-hvac</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr"/>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Oakridge principal and APS Facilities</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>What is the interim plan for hot classrooms between now and the summer 2027 construction start?</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>The April 2026 email asked this for one spring. The reply named who would monitor, not what would be done.</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr"/>
+      <c r="H4" s="2" t="inlineStr"/>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
         <is>
           <t>email-2026-04</t>
         </is>
@@ -2249,10 +2984,10 @@
     <dataValidation sqref="B2:B500" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Unknown reference" error="Must match an id already listed on Needs" type="list">
       <formula1>=Needs!$A$2:$A$500</formula1>
     </dataValidation>
-    <dataValidation sqref="H2:H500" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Not an allowed value" error="Use one of: answered, partial, unanswered" type="list">
-      <formula1>"answered,partial,unanswered"</formula1>
+    <dataValidation sqref="I2:I500" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Not an allowed value" error="Use one of: open, answered, partial, unanswered" type="list">
+      <formula1>"open,answered,partial,unanswered"</formula1>
     </dataValidation>
-    <dataValidation sqref="I2:I500" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Unknown reference" error="Must match an id already listed on Sources" type="list">
+    <dataValidation sqref="J2:J500" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Unknown reference" error="Must match an id already listed on Sources" type="list">
       <formula1>=Sources!$A$2:$A$500</formula1>
     </dataValidation>
   </dataValidations>
@@ -2266,358 +3001,186 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:H4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="24" customWidth="1" min="1" max="1"/>
-    <col width="60" customWidth="1" min="2" max="2"/>
-    <col width="51" customWidth="1" min="3" max="3"/>
-    <col width="60" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="60" customWidth="1" min="6" max="6"/>
+    <col width="21" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="60" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="59" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
+          <t>funding_id</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>need_id</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>label</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>amount</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>parent_id</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>note</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>basis</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
           <t>source_id</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>title</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>publisher</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>url</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>retrieved_on</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>notes</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>cip-fy27-36</t>
+          <t>q4-bond</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>APS Approved FY 2027-36 Capital Improvement Plan (CIP)</t>
+          <t>oakridge-hvac</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Arlington Public Schools</t>
+          <t>Question 4: school bond on the Nov 3, 2026 ballot</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>https://www.apsva.us/wp-content/uploads/sites/57/2026/08/APS-FY2027-36-CIP-REPORT-FINAL.pdf</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>Adopted June 18 2026; report dated August 2026; Appendix C funding timeline is an image (not read)</t>
+          <t>80000000</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr"/>
+      <c r="F2" s="2" t="inlineStr"/>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>fact</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>county-bond-2026</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>aps-cip-approval-post</t>
+          <t>oakridge-refresh</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>School Board Approves FY 2027-36 CIP Focused on School Renewal and Modernization</t>
+          <t>oakridge-hvac</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Arlington Public Schools</t>
+          <t>Oakridge Elementary Refresh (HVAC, roofing, flooring, painting)</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>https://www.apsva.us/post/school-board-approves-fy-2027-36-cip-focused-on-school-renewal-and-modernization/</t>
+          <t>31000000</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
-      <c r="F3" s="2" t="inlineStr">
-        <is>
-          <t>News post June 19 2026</t>
+          <t>q4-bond</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr"/>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>estimate</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>cip-fy27-36</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>aps-engage-cip</t>
+          <t>oakridge-hvac-slice</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>FY 2027-36 Capital Improvement Plan</t>
+          <t>oakridge-hvac</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Arlington Public Schools</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>https://www.apsva.us/engage/cip/</t>
-        </is>
-      </c>
+          <t>HVAC replacement</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr"/>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>oakridge-refresh</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Lists Election Day as Nov 4 (conflicts with Nov 3 elsewhere)</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>county-bond-2026</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>2026 Bond Referenda</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>Arlington County Government</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>https://www.arlingtonva.us/Government/Programs/Budget-Finance/Bonds/2026-Bond-Referenda</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
-      <c r="F5" s="2" t="inlineStr">
-        <is>
-          <t>Question 4 text and project list</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>policy-d15-draft-2025</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>Proposed revisions to Policy D-15 External Funding-Commercial Activities (draft)</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>Arlington School Board (BoardDocs)</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>https://go.boarddocs.com/vsba/arlington/Board.nsf/files/DD8P9T6391D5/$file/D-15%20External%20Funding-Commercial%20Activities.pdf</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
-      <c r="F6" s="2" t="inlineStr">
-        <is>
-          <t>January 2025 first draft; adopted text not verified</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>aps-budget-page</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>Budget</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>Arlington Public Schools</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="inlineStr">
-        <is>
-          <t>https://www.apsva.us/budget/</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
-      <c r="F7" s="2" t="inlineStr">
-        <is>
-          <t>FY27 MC/MM $3.0M one-time; no definition</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>aps-superintendent</t>
-        </is>
-      </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>Superintendent's Office</t>
-        </is>
-      </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>Arlington Public Schools</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="inlineStr">
-        <is>
-          <t>https://www.apsva.us/departments/superintendents-office/</t>
-        </is>
-      </c>
-      <c r="E8" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
-      <c r="F8" s="2" t="inlineStr"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>aps-sign-up-to-speak</t>
-        </is>
-      </c>
-      <c r="B9" s="2" t="inlineStr">
-        <is>
-          <t>Speak at a School Board Meeting</t>
-        </is>
-      </c>
-      <c r="C9" s="2" t="inlineStr">
-        <is>
-          <t>Arlington Public Schools</t>
-        </is>
-      </c>
-      <c r="D9" s="2" t="inlineStr">
-        <is>
-          <t>https://www.apsva.us/arlington-school-board/school-board-meetings/sign-up-to-speak/</t>
-        </is>
-      </c>
-      <c r="E9" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
-      <c r="F9" s="2" t="inlineStr"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>aps-sept-2026-schedule</t>
-        </is>
-      </c>
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>September Schedule of Board Meetings Work Sessions and Advisory Council and Committee Meetings</t>
-        </is>
-      </c>
-      <c r="C10" s="2" t="inlineStr">
-        <is>
-          <t>Arlington Public Schools</t>
-        </is>
-      </c>
-      <c r="D10" s="2" t="inlineStr">
-        <is>
-          <t>https://www.apsva.us/post/september-schedule-of-board-meetings-work-sessions-and-advisory-council-and-committee-meetings-4/</t>
-        </is>
-      </c>
-      <c r="E10" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
-      <c r="F10" s="2" t="inlineStr">
-        <is>
-          <t>Posted Sep 2 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t>email-2026-04</t>
-        </is>
-      </c>
-      <c r="B11" s="2" t="inlineStr">
-        <is>
-          <t>Email exchange with Superintendent Durán, April 15–16 2026</t>
-        </is>
-      </c>
-      <c r="C11" s="2" t="inlineStr">
-        <is>
-          <t>Provided by team member (personal correspondence)</t>
-        </is>
-      </c>
-      <c r="D11" s="2" t="inlineStr"/>
-      <c r="E11" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
-      <c r="F11" s="2" t="inlineStr">
-        <is>
-          <t>Original held by the team; quoted in the pitch video.</t>
+          <t>No APS or County document prices the HVAC work by itself.</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>interpretation</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>cip-fy27-36</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <dataValidations count="4">
+    <dataValidation sqref="B2:B500" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Unknown reference" error="Must match an id already listed on Needs" type="list">
+      <formula1>=Needs!$A$2:$A$500</formula1>
+    </dataValidation>
+    <dataValidation sqref="E2:E500" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Unknown reference" error="Must match an id already listed on Funding" type="list">
+      <formula1>=Funding!$A$2:$A$500</formula1>
+    </dataValidation>
+    <dataValidation sqref="G2:G500" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Not an allowed value" error="Use one of: fact, requirement, estimate, interpretation" type="list">
+      <formula1>"fact,requirement,estimate,interpretation"</formula1>
+    </dataValidation>
+    <dataValidation sqref="H2:H500" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Unknown reference" error="Must match an id already listed on Sources" type="list">
+      <formula1>=Sources!$A$2:$A$500</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2628,346 +3191,420 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D16"/>
+  <dimension ref="A1:F13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="41" customWidth="1" min="2" max="2"/>
-    <col width="60" customWidth="1" min="3" max="3"/>
-    <col width="48" customWidth="1" min="4" max="4"/>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="60" customWidth="1" min="2" max="2"/>
+    <col width="51" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="60" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>tab</t>
+          <t>source_id</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>column</t>
+          <t>title</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>meaning</t>
+          <t>publisher</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>allowed_values</t>
+          <t>url</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>retrieved_on</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>notes</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Tracks</t>
+          <t>cip-fy27-36</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>track_id</t>
+          <t>APS Approved FY 2027-36 Capital Improvement Plan (CIP)</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Short id for the track (lowercase-dashes)</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr"/>
+          <t>Arlington Public Schools</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>https://www.apsva.us/wp-content/uploads/sites/57/2026/08/APS-FY2027-36-CIP-REPORT-FINAL.pdf</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Adopted June 18 2026; report dated August 2026; Appendix C funding timeline is an image (not read)</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Tracks</t>
+          <t>aps-cip-approval-post</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>verification</t>
+          <t>School Board Approves FY 2027-36 CIP Focused on School Renewal and Modernization</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Has an APS contact confirmed this track's stages and deciders?</t>
+          <t>Arlington Public Schools</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>draft | documented | confirmed</t>
+          <t>https://www.apsva.us/post/school-board-approves-fy-2027-36-cip-focused-on-school-renewal-and-modernization/</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>News post June 19 2026</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Stages</t>
+          <t>aps-engage-cip</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>order</t>
+          <t>FY 2027-36 Capital Improvement Plan</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Position of the stage within its track (1 = first)</t>
+          <t>Arlington Public Schools</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>whole number</t>
+          <t>https://www.apsva.us/engage/cip/</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>Lists Election Day as Nov 4 (conflicts with Nov 3 elsewhere)</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Stages</t>
+          <t>county-bond-2026</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>basis</t>
+          <t>2026 Bond Referenda</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>What kind of claim the stage is</t>
+          <t>Arlington County Government</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>fact | requirement | estimate | interpretation</t>
+          <t>https://www.arlingtonva.us/Government/Programs/Budget-Finance/Bonds/2026-Bond-Referenda</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>Question 4 text and project list</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Schools</t>
+          <t>policy-d15-draft-2025</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>status</t>
+          <t>Proposed revisions to Policy D-15 External Funding-Commercial Activities (draft)</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>live = every claim must have a source or the site will not build; draft = warnings only</t>
+          <t>Arlington School Board (BoardDocs)</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>live | draft</t>
+          <t>https://go.boarddocs.com/vsba/arlington/Board.nsf/files/DD8P9T6391D5/$file/D-15%20External%20Funding-Commercial%20Activities.pdf</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>January 2025 first draft; adopted text not verified</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Needs</t>
+          <t>aps-budget-page</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>current_stage_id</t>
+          <t>Budget</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Must be a stage_id that belongs to the need's track_id</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="inlineStr"/>
+          <t>Arlington Public Schools</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>https://www.apsva.us/budget/</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>FY27 MC/MM $3.0M one-time; no definition</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Needs</t>
+          <t>aps-superintendent</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>stage_basis / cost_basis / window_basis</t>
+          <t>Superintendent's Office</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>What kind of claim each is</t>
+          <t>Arlington Public Schools</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>fact | requirement | estimate | interpretation</t>
-        </is>
-      </c>
+          <t>https://www.apsva.us/departments/superintendents-office/</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Milestones</t>
+          <t>aps-sign-up-to-speak</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>status</t>
+          <t>Speak at a School Board Meeting</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Exactly one milestone per need must be next</t>
+          <t>Arlington Public Schools</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>done | next | later</t>
-        </is>
-      </c>
+          <t>https://www.apsva.us/arlington-school-board/school-board-meetings/sign-up-to-speak/</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Milestones</t>
+          <t>aps-sept-2026-schedule</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>basis</t>
+          <t>September Schedule of Board Meetings Work Sessions and Advisory Council and Committee Meetings</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>What kind of claim the milestone is</t>
+          <t>Arlington Public Schools</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>fact | requirement | estimate | interpretation</t>
+          <t>https://www.apsva.us/post/september-schedule-of-board-meetings-work-sessions-and-advisory-council-and-committee-meetings-4/</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>Posted Sep 2 2026</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Milestones</t>
+          <t>email-2026-04</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>date</t>
+          <t>Email exchange with Superintendent Durán, April 15–16 2026</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>ISO date</t>
-        </is>
-      </c>
-      <c r="D11" s="2" t="inlineStr">
-        <is>
-          <t>YYYY-MM-DD</t>
+          <t>Provided by team member (personal correspondence)</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr"/>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>Original held by the team; quoted in the pitch video.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Engage</t>
+          <t>aps-sb-meetings-2026-27</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>basis</t>
+          <t>School Board Meetings (2026-27 dates)</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>What kind of claim the venue is</t>
+          <t>Arlington Public Schools</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>fact | requirement | estimate | interpretation</t>
+          <t>https://www.apsva.us/arlington-school-board/school-board-meetings/</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>Lists Oct 8, Oct 22, Nov 12 2026; 7 p.m. at Syphax unless noted</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Inquiries</t>
+          <t>ccpta-2026-27</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>status</t>
+          <t>Arlington County Council of PTAs: 2026-27 meetings</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Did the authority answer the question?</t>
+          <t>Arlington CCPTA</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>answered | partial | unanswered</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="2" t="inlineStr">
-        <is>
-          <t>Sources</t>
-        </is>
-      </c>
-      <c r="B14" s="2" t="inlineStr">
-        <is>
-          <t>source_id</t>
-        </is>
-      </c>
-      <c r="C14" s="2" t="inlineStr">
-        <is>
-          <t>Referenced by every *_source_id column. Add the document here first.</t>
-        </is>
-      </c>
-      <c r="D14" s="2" t="inlineStr"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="2" t="inlineStr">
-        <is>
-          <t>(all)</t>
-        </is>
-      </c>
-      <c r="B15" s="2" t="inlineStr">
-        <is>
-          <t>*_id</t>
-        </is>
-      </c>
-      <c r="C15" s="2" t="inlineStr">
-        <is>
-          <t>Lowercase letters and digits and dashes only. No spaces.</t>
-        </is>
-      </c>
-      <c r="D15" s="2" t="inlineStr"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="2" t="inlineStr">
-        <is>
-          <t>(all)</t>
-        </is>
-      </c>
-      <c r="B16" s="2" t="inlineStr">
-        <is>
-          <t>blank cell</t>
-        </is>
-      </c>
-      <c r="C16" s="2" t="inlineStr">
-        <is>
-          <t>Leave blank when unknown. Never type TBD or ?.</t>
-        </is>
-      </c>
-      <c r="D16" s="2" t="inlineStr"/>
+          <t>https://www.arlingtonccpta.org/</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>Zoom, 7 p.m.; open to PTA delegates and executive board invitees only</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>